<commit_message>
make some changes to the trip changes and its % valie distribution
</commit_message>
<xml_diff>
--- a/Viajante/Volume_por_rota.xlsx
+++ b/Viajante/Volume_por_rota.xlsx
@@ -76,7 +76,7 @@
     <t>% MDRs APURADOS</t>
   </si>
   <si>
-    <t>FCA</t>
+    <t>FPT</t>
   </si>
   <si>
     <t>Apr</t>
@@ -115,25 +115,25 @@
     <t>Sep</t>
   </si>
   <si>
-    <t>800006503</t>
-  </si>
-  <si>
-    <t>COOPER STANDARD III</t>
+    <t>800033128</t>
+  </si>
+  <si>
+    <t>MAHLE</t>
   </si>
   <si>
     <t>CARRETA SIDER</t>
   </si>
   <si>
-    <t>MONTAGEM-MG</t>
+    <t>MONTAGEM-SP</t>
   </si>
   <si>
     <t>FTL</t>
   </si>
   <si>
-    <t>FURLONG</t>
-  </si>
-  <si>
-    <t>VOLUME</t>
+    <t>JSL</t>
+  </si>
+  <si>
+    <t>PESO</t>
   </si>
   <si>
     <t>Alterar último veículo para menor porte</t>
@@ -564,7 +564,7 @@
     </row>
     <row r="2" spans="1:20">
       <c r="A2">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B2">
         <v>1080</v>
@@ -597,25 +597,25 @@
         <v>39</v>
       </c>
       <c r="L2">
-        <v>503.8</v>
+        <v>61349.1</v>
       </c>
       <c r="M2">
-        <v>47721.8</v>
+        <v>5735796.7</v>
       </c>
       <c r="N2">
-        <v>649</v>
+        <v>24278</v>
       </c>
       <c r="O2">
-        <v>636.1799999999999</v>
+        <v>22943.16</v>
       </c>
       <c r="P2">
-        <v>7</v>
+        <v>230</v>
       </c>
       <c r="Q2">
-        <v>72</v>
+        <v>266.7</v>
       </c>
       <c r="R2">
-        <v>90.88</v>
+        <v>99.75</v>
       </c>
       <c r="S2" t="s">
         <v>40</v>
@@ -626,7 +626,7 @@
     </row>
     <row r="3" spans="1:20">
       <c r="A3">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B3">
         <v>1080</v>
@@ -659,28 +659,28 @@
         <v>39</v>
       </c>
       <c r="L3">
-        <v>818.7</v>
+        <v>97221.10000000001</v>
       </c>
       <c r="M3">
-        <v>77544.39999999999</v>
+        <v>9165920.699999999</v>
       </c>
       <c r="N3">
-        <v>1051</v>
+        <v>38460</v>
       </c>
       <c r="O3">
-        <v>1032.78</v>
+        <v>36663.71</v>
       </c>
       <c r="P3">
-        <v>11</v>
+        <v>367</v>
       </c>
       <c r="Q3">
-        <v>74.40000000000001</v>
+        <v>264.9</v>
       </c>
       <c r="R3">
-        <v>93.89</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="S3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T3">
         <v>100</v>
@@ -688,7 +688,7 @@
     </row>
     <row r="4" spans="1:20">
       <c r="A4">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B4">
         <v>1080</v>
@@ -721,25 +721,25 @@
         <v>39</v>
       </c>
       <c r="L4">
-        <v>526.8</v>
+        <v>46822</v>
       </c>
       <c r="M4">
-        <v>49510.2</v>
+        <v>4673839.4</v>
       </c>
       <c r="N4">
-        <v>678</v>
+        <v>20163</v>
       </c>
       <c r="O4">
-        <v>664.9400000000001</v>
+        <v>18695.35</v>
       </c>
       <c r="P4">
-        <v>7</v>
+        <v>187</v>
       </c>
       <c r="Q4">
-        <v>75.3</v>
+        <v>250.4</v>
       </c>
       <c r="R4">
-        <v>94.98999999999999</v>
+        <v>99.98</v>
       </c>
       <c r="S4" t="s">
         <v>41</v>
@@ -750,7 +750,7 @@
     </row>
     <row r="5" spans="1:20">
       <c r="A5">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B5">
         <v>1080</v>
@@ -783,25 +783,25 @@
         <v>39</v>
       </c>
       <c r="L5">
-        <v>418.6</v>
+        <v>51311.8</v>
       </c>
       <c r="M5">
-        <v>39559.5</v>
+        <v>4807560</v>
       </c>
       <c r="N5">
-        <v>537</v>
+        <v>19774</v>
       </c>
       <c r="O5">
-        <v>528.03</v>
+        <v>19230.23</v>
       </c>
       <c r="P5">
-        <v>6</v>
+        <v>193</v>
       </c>
       <c r="Q5">
-        <v>69.8</v>
+        <v>265.9</v>
       </c>
       <c r="R5">
-        <v>88</v>
+        <v>99.64</v>
       </c>
       <c r="S5" t="s">
         <v>40</v>
@@ -812,7 +812,7 @@
     </row>
     <row r="6" spans="1:20">
       <c r="A6">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B6">
         <v>1080</v>
@@ -845,25 +845,25 @@
         <v>39</v>
       </c>
       <c r="L6">
-        <v>621.7</v>
+        <v>53063.5</v>
       </c>
       <c r="M6">
-        <v>58893.9</v>
+        <v>5417696.2</v>
       </c>
       <c r="N6">
-        <v>800</v>
+        <v>22889</v>
       </c>
       <c r="O6">
-        <v>784.74</v>
+        <v>21670.81</v>
       </c>
       <c r="P6">
-        <v>8</v>
+        <v>217</v>
       </c>
       <c r="Q6">
-        <v>77.7</v>
+        <v>244.5</v>
       </c>
       <c r="R6">
-        <v>98.09</v>
+        <v>99.87</v>
       </c>
       <c r="S6" t="s">
         <v>41</v>
@@ -874,7 +874,7 @@
     </row>
     <row r="7" spans="1:20">
       <c r="A7">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B7">
         <v>1080</v>
@@ -907,28 +907,28 @@
         <v>39</v>
       </c>
       <c r="L7">
-        <v>570.7</v>
+        <v>71434.10000000001</v>
       </c>
       <c r="M7">
-        <v>54442.7</v>
+        <v>6690972</v>
       </c>
       <c r="N7">
-        <v>736</v>
+        <v>27704</v>
       </c>
       <c r="O7">
-        <v>720.67</v>
+        <v>26763.87</v>
       </c>
       <c r="P7">
-        <v>8</v>
+        <v>268</v>
       </c>
       <c r="Q7">
-        <v>71.3</v>
+        <v>266.5</v>
       </c>
       <c r="R7">
-        <v>90.08</v>
+        <v>99.87</v>
       </c>
       <c r="S7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T7">
         <v>100</v>
@@ -936,7 +936,7 @@
     </row>
     <row r="8" spans="1:20">
       <c r="A8">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B8">
         <v>1080</v>
@@ -969,28 +969,28 @@
         <v>39</v>
       </c>
       <c r="L8">
-        <v>527</v>
+        <v>66432.2</v>
       </c>
       <c r="M8">
-        <v>49724.4</v>
+        <v>6186255.5</v>
       </c>
       <c r="N8">
-        <v>680</v>
+        <v>25888</v>
       </c>
       <c r="O8">
-        <v>665.78</v>
+        <v>24745.01</v>
       </c>
       <c r="P8">
-        <v>7</v>
+        <v>248</v>
       </c>
       <c r="Q8">
-        <v>75.3</v>
+        <v>267.9</v>
       </c>
       <c r="R8">
-        <v>95.11</v>
+        <v>99.78</v>
       </c>
       <c r="S8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T8">
         <v>100</v>
@@ -998,7 +998,7 @@
     </row>
     <row r="9" spans="1:20">
       <c r="A9">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B9">
         <v>1080</v>
@@ -1031,28 +1031,28 @@
         <v>39</v>
       </c>
       <c r="L9">
-        <v>719.9</v>
+        <v>88054.7</v>
       </c>
       <c r="M9">
-        <v>68327.7</v>
+        <v>8240045.1</v>
       </c>
       <c r="N9">
-        <v>928</v>
+        <v>34563</v>
       </c>
       <c r="O9">
-        <v>909.42</v>
+        <v>32960.2</v>
       </c>
       <c r="P9">
-        <v>10</v>
+        <v>330</v>
       </c>
       <c r="Q9">
-        <v>72</v>
+        <v>266.8</v>
       </c>
       <c r="R9">
-        <v>90.94</v>
+        <v>99.88</v>
       </c>
       <c r="S9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T9">
         <v>100</v>
@@ -1060,7 +1060,7 @@
     </row>
     <row r="10" spans="1:20">
       <c r="A10">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B10">
         <v>1080</v>
@@ -1093,25 +1093,25 @@
         <v>39</v>
       </c>
       <c r="L10">
-        <v>736.6</v>
+        <v>93571.3</v>
       </c>
       <c r="M10">
-        <v>70150.3</v>
+        <v>8777739.4</v>
       </c>
       <c r="N10">
-        <v>950</v>
+        <v>36388</v>
       </c>
       <c r="O10">
-        <v>930.28</v>
+        <v>35110.95</v>
       </c>
       <c r="P10">
-        <v>10</v>
+        <v>352</v>
       </c>
       <c r="Q10">
-        <v>73.7</v>
+        <v>265.8</v>
       </c>
       <c r="R10">
-        <v>93.03</v>
+        <v>99.75</v>
       </c>
       <c r="S10" t="s">
         <v>40</v>
@@ -1122,7 +1122,7 @@
     </row>
     <row r="11" spans="1:20">
       <c r="A11">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B11">
         <v>1080</v>
@@ -1155,25 +1155,25 @@
         <v>39</v>
       </c>
       <c r="L11">
-        <v>747.2</v>
+        <v>66899.2</v>
       </c>
       <c r="M11">
-        <v>71169.7</v>
+        <v>6678461</v>
       </c>
       <c r="N11">
-        <v>961</v>
+        <v>28996</v>
       </c>
       <c r="O11">
-        <v>942.74</v>
+        <v>26713.85</v>
       </c>
       <c r="P11">
-        <v>10</v>
+        <v>268</v>
       </c>
       <c r="Q11">
-        <v>74.7</v>
+        <v>249.6</v>
       </c>
       <c r="R11">
-        <v>94.27</v>
+        <v>99.68000000000001</v>
       </c>
       <c r="S11" t="s">
         <v>40</v>
@@ -1184,7 +1184,7 @@
     </row>
     <row r="12" spans="1:20">
       <c r="A12">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B12">
         <v>1080</v>
@@ -1217,28 +1217,28 @@
         <v>39</v>
       </c>
       <c r="L12">
-        <v>637.1</v>
+        <v>63200.7</v>
       </c>
       <c r="M12">
-        <v>60577.4</v>
+        <v>6195728.9</v>
       </c>
       <c r="N12">
-        <v>823</v>
+        <v>26406</v>
       </c>
       <c r="O12">
-        <v>805.1900000000001</v>
+        <v>24782.88</v>
       </c>
       <c r="P12">
-        <v>9</v>
+        <v>248</v>
       </c>
       <c r="Q12">
-        <v>70.8</v>
+        <v>254.8</v>
       </c>
       <c r="R12">
-        <v>89.47</v>
+        <v>99.93000000000001</v>
       </c>
       <c r="S12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T12">
         <v>100</v>
@@ -1246,7 +1246,7 @@
     </row>
     <row r="13" spans="1:20">
       <c r="A13">
-        <v>22</v>
+        <v>160</v>
       </c>
       <c r="B13">
         <v>1080</v>
@@ -1279,28 +1279,28 @@
         <v>39</v>
       </c>
       <c r="L13">
-        <v>612.2</v>
+        <v>67708.2</v>
       </c>
       <c r="M13">
-        <v>57665.5</v>
+        <v>6506613.6</v>
       </c>
       <c r="N13">
-        <v>791</v>
+        <v>27301</v>
       </c>
       <c r="O13">
-        <v>773.72</v>
+        <v>26026.47</v>
       </c>
       <c r="P13">
-        <v>8</v>
+        <v>261</v>
       </c>
       <c r="Q13">
-        <v>76.5</v>
+        <v>259.4</v>
       </c>
       <c r="R13">
-        <v>96.72</v>
+        <v>99.72</v>
       </c>
       <c r="S13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="T13">
         <v>100</v>

</xml_diff>